<commit_message>
feat(catalog): restore 100% authentic 59 Pasalubong raw materials and 28 finished products with exact BOM linkages
</commit_message>
<xml_diff>
--- a/DATASETS/ACTUAL_DATA_2026_YTD/RMIMS_59_RAW_MATERIALS_CATALOG.xlsx
+++ b/DATASETS/ACTUAL_DATA_2026_YTD/RMIMS_59_RAW_MATERIALS_CATALOG.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H60"/>
+  <dimension ref="A1:I60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -429,30 +429,35 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
           <t>unit_of_measure</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>current_stock</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>minimum_threshold</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>reorder_quantity</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>lead_time_days</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>shortage_status</t>
         </is>
@@ -466,29 +471,34 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Bread Flour</t>
+          <t>Food Grade Sunset Yellow / Orange Dye</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
-        <v>144</v>
+          <t>Additives &amp; Colors</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
       </c>
       <c r="E2" t="n">
-        <v>200</v>
+        <v>22</v>
       </c>
       <c r="F2" t="n">
-        <v>420</v>
+        <v>10</v>
       </c>
       <c r="G2" t="n">
-        <v>3</v>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>LOW STOCK</t>
+        <v>25</v>
+      </c>
+      <c r="H2" t="n">
+        <v>5</v>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>IN STOCK</t>
         </is>
       </c>
     </row>
@@ -500,27 +510,32 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>All-Purpose Flour</t>
+          <t>Baking Powder</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="D3" t="n">
-        <v>345</v>
+          <t>Baking Supplies</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
       </c>
       <c r="E3" t="n">
-        <v>160</v>
+        <v>55</v>
       </c>
       <c r="F3" t="n">
-        <v>350</v>
+        <v>25</v>
       </c>
       <c r="G3" t="n">
+        <v>50</v>
+      </c>
+      <c r="H3" t="n">
         <v>3</v>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>IN STOCK</t>
         </is>
@@ -534,27 +549,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Cake Flour</t>
+          <t>Cream of Tartar</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="D4" t="n">
-        <v>74</v>
+          <t>Baking Supplies</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
       </c>
       <c r="E4" t="n">
-        <v>100</v>
+        <v>10</v>
       </c>
       <c r="F4" t="n">
-        <v>220</v>
+        <v>10</v>
       </c>
       <c r="G4" t="n">
+        <v>20</v>
+      </c>
+      <c r="H4" t="n">
         <v>4</v>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>LOW STOCK</t>
         </is>
@@ -568,27 +588,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Refined White Sugar</t>
+          <t>Instant Dry Yeast</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="D5" t="n">
-        <v>133</v>
+          <t>Baking Supplies</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
       </c>
       <c r="E5" t="n">
-        <v>180</v>
+        <v>18</v>
       </c>
       <c r="F5" t="n">
-        <v>380</v>
+        <v>20</v>
       </c>
       <c r="G5" t="n">
-        <v>2</v>
-      </c>
-      <c r="H5" t="inlineStr">
+        <v>40</v>
+      </c>
+      <c r="H5" t="n">
+        <v>3</v>
+      </c>
+      <c r="I5" t="inlineStr">
         <is>
           <t>LOW STOCK</t>
         </is>
@@ -602,27 +627,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Brown Sugar</t>
+          <t>Cane Vinegar</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="D6" t="n">
+          <t>Condiments &amp; Acids</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
         <v>176</v>
       </c>
-      <c r="E6" t="n">
+      <c r="F6" t="n">
         <v>80</v>
       </c>
-      <c r="F6" t="n">
-        <v>180</v>
-      </c>
       <c r="G6" t="n">
-        <v>3</v>
-      </c>
-      <c r="H6" t="inlineStr">
+        <v>150</v>
+      </c>
+      <c r="H6" t="n">
+        <v>4</v>
+      </c>
+      <c r="I6" t="inlineStr">
         <is>
           <t>IN STOCK</t>
         </is>
@@ -636,29 +666,34 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Powdered Sugar (Icing)</t>
+          <t>Soy Sauce</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="D7" t="n">
-        <v>43</v>
+          <t>Condiments &amp; Acids</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
       </c>
       <c r="E7" t="n">
+        <v>134</v>
+      </c>
+      <c r="F7" t="n">
         <v>60</v>
       </c>
-      <c r="F7" t="n">
-        <v>140</v>
-      </c>
       <c r="G7" t="n">
-        <v>3</v>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>LOW STOCK</t>
+        <v>120</v>
+      </c>
+      <c r="H7" t="n">
+        <v>4</v>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>IN STOCK</t>
         </is>
       </c>
     </row>
@@ -670,27 +705,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Unsalted Butter</t>
+          <t>Condensed Milk</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="D8" t="n">
-        <v>87</v>
+          <t>Dairy</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
       </c>
       <c r="E8" t="n">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="F8" t="n">
-        <v>280</v>
+        <v>150</v>
       </c>
       <c r="G8" t="n">
-        <v>2</v>
-      </c>
-      <c r="H8" t="inlineStr">
+        <v>300</v>
+      </c>
+      <c r="H8" t="n">
+        <v>3</v>
+      </c>
+      <c r="I8" t="inlineStr">
         <is>
           <t>LOW STOCK</t>
         </is>
@@ -704,27 +744,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Salted Butter</t>
+          <t>Evaporated Milk</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="D9" t="n">
-        <v>158</v>
+          <t>Dairy</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
       </c>
       <c r="E9" t="n">
-        <v>70</v>
+        <v>259</v>
       </c>
       <c r="F9" t="n">
-        <v>160</v>
+        <v>120</v>
       </c>
       <c r="G9" t="n">
-        <v>2</v>
-      </c>
-      <c r="H9" t="inlineStr">
+        <v>250</v>
+      </c>
+      <c r="H9" t="n">
+        <v>3</v>
+      </c>
+      <c r="I9" t="inlineStr">
         <is>
           <t>IN STOCK</t>
         </is>
@@ -738,27 +783,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Margarine</t>
+          <t>Powdered Milk</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="D10" t="n">
-        <v>194</v>
+          <t>Dairy</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
       </c>
       <c r="E10" t="n">
-        <v>90</v>
+        <v>432</v>
       </c>
       <c r="F10" t="n">
-        <v>230</v>
+        <v>200</v>
       </c>
       <c r="G10" t="n">
-        <v>3</v>
-      </c>
-      <c r="H10" t="inlineStr">
+        <v>400</v>
+      </c>
+      <c r="H10" t="n">
+        <v>4</v>
+      </c>
+      <c r="I10" t="inlineStr">
         <is>
           <t>IN STOCK</t>
         </is>
@@ -772,27 +822,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Vegetable Shortening</t>
+          <t>Fresh Whole Egg Whites</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="D11" t="n">
-        <v>62</v>
+          <t>Dairy &amp; Eggs</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
       </c>
       <c r="E11" t="n">
-        <v>80</v>
+        <v>57</v>
       </c>
       <c r="F11" t="n">
-        <v>190</v>
+        <v>75</v>
       </c>
       <c r="G11" t="n">
-        <v>4</v>
-      </c>
-      <c r="H11" t="inlineStr">
+        <v>150</v>
+      </c>
+      <c r="H11" t="n">
+        <v>2</v>
+      </c>
+      <c r="I11" t="inlineStr">
         <is>
           <t>LOW STOCK</t>
         </is>
@@ -806,29 +861,34 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Pasteurized Whole Eggs</t>
+          <t>Fresh Whole Eggs</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="D12" t="n">
-        <v>94</v>
+          <t>Dairy &amp; Eggs</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
       </c>
       <c r="E12" t="n">
-        <v>130</v>
+        <v>542</v>
       </c>
       <c r="F12" t="n">
-        <v>320</v>
+        <v>250</v>
       </c>
       <c r="G12" t="n">
-        <v>1</v>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>LOW STOCK</t>
+        <v>500</v>
+      </c>
+      <c r="H12" t="n">
+        <v>2</v>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>IN STOCK</t>
         </is>
       </c>
     </row>
@@ -840,27 +900,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Egg Yolks (Liquid)</t>
+          <t>All-Vegetable Shortening</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="D13" t="n">
-        <v>111</v>
+          <t>Dairy &amp; Fats</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
       </c>
       <c r="E13" t="n">
-        <v>50</v>
+        <v>220</v>
       </c>
       <c r="F13" t="n">
-        <v>130</v>
+        <v>100</v>
       </c>
       <c r="G13" t="n">
-        <v>2</v>
-      </c>
-      <c r="H13" t="inlineStr">
+        <v>200</v>
+      </c>
+      <c r="H13" t="n">
+        <v>5</v>
+      </c>
+      <c r="I13" t="inlineStr">
         <is>
           <t>IN STOCK</t>
         </is>
@@ -874,27 +939,32 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Egg Whites (Liquid)</t>
+          <t>Baking Shortening</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="D14" t="n">
-        <v>34</v>
+          <t>Dairy &amp; Fats</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
       </c>
       <c r="E14" t="n">
-        <v>45</v>
+        <v>75</v>
       </c>
       <c r="F14" t="n">
-        <v>110</v>
+        <v>100</v>
       </c>
       <c r="G14" t="n">
-        <v>2</v>
-      </c>
-      <c r="H14" t="inlineStr">
+        <v>200</v>
+      </c>
+      <c r="H14" t="n">
+        <v>5</v>
+      </c>
+      <c r="I14" t="inlineStr">
         <is>
           <t>LOW STOCK</t>
         </is>
@@ -908,27 +978,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Full Cream Milk</t>
+          <t>Salted Creamery Butter</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="D15" t="n">
-        <v>75</v>
+          <t>Dairy &amp; Fats</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
       </c>
       <c r="E15" t="n">
-        <v>100</v>
+        <v>69</v>
       </c>
       <c r="F15" t="n">
-        <v>250</v>
+        <v>90</v>
       </c>
       <c r="G15" t="n">
-        <v>2</v>
-      </c>
-      <c r="H15" t="inlineStr">
+        <v>180</v>
+      </c>
+      <c r="H15" t="n">
+        <v>4</v>
+      </c>
+      <c r="I15" t="inlineStr">
         <is>
           <t>LOW STOCK</t>
         </is>
@@ -942,27 +1017,32 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Skimmed Milk Powder</t>
+          <t>Seedless Raisins</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="D16" t="n">
-        <v>135</v>
+          <t>Dry Goods</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
       </c>
       <c r="E16" t="n">
-        <v>60</v>
+        <v>88</v>
       </c>
       <c r="F16" t="n">
-        <v>150</v>
+        <v>40</v>
       </c>
       <c r="G16" t="n">
-        <v>4</v>
-      </c>
-      <c r="H16" t="inlineStr">
+        <v>80</v>
+      </c>
+      <c r="H16" t="n">
+        <v>7</v>
+      </c>
+      <c r="I16" t="inlineStr">
         <is>
           <t>IN STOCK</t>
         </is>
@@ -976,27 +1056,32 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Evaporated Milk</t>
+          <t>Vanilla Extract</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
+          <t>Flavorings &amp; Extracts</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
           <t>L</t>
         </is>
       </c>
-      <c r="D17" t="n">
-        <v>158</v>
-      </c>
       <c r="E17" t="n">
-        <v>70</v>
+        <v>25</v>
       </c>
       <c r="F17" t="n">
-        <v>170</v>
+        <v>10</v>
       </c>
       <c r="G17" t="n">
-        <v>3</v>
-      </c>
-      <c r="H17" t="inlineStr">
+        <v>20</v>
+      </c>
+      <c r="H17" t="n">
+        <v>6</v>
+      </c>
+      <c r="I17" t="inlineStr">
         <is>
           <t>IN STOCK</t>
         </is>
@@ -1010,29 +1095,34 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Condensed Milk</t>
+          <t>All-Purpose Wheat Flour</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="D18" t="n">
-        <v>59</v>
+          <t>Grains &amp; Flours</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
       </c>
       <c r="E18" t="n">
-        <v>80</v>
+        <v>1294</v>
       </c>
       <c r="F18" t="n">
-        <v>200</v>
+        <v>600</v>
       </c>
       <c r="G18" t="n">
+        <v>1200</v>
+      </c>
+      <c r="H18" t="n">
         <v>3</v>
       </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>LOW STOCK</t>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>IN STOCK</t>
         </is>
       </c>
     </row>
@@ -1044,29 +1134,34 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Heavy Whipping Cream</t>
+          <t>Cornstarch</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="D19" t="n">
-        <v>49</v>
+          <t>Grains &amp; Flours</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
       </c>
       <c r="E19" t="n">
-        <v>65</v>
+        <v>328</v>
       </c>
       <c r="F19" t="n">
         <v>150</v>
       </c>
       <c r="G19" t="n">
-        <v>2</v>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>LOW STOCK</t>
+        <v>300</v>
+      </c>
+      <c r="H19" t="n">
+        <v>4</v>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>IN STOCK</t>
         </is>
       </c>
     </row>
@@ -1078,29 +1173,34 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Instant Dry Yeast</t>
+          <t>Glutinous Rice (Malagkit for Pinipig)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="D20" t="n">
-        <v>21</v>
+          <t>Grains &amp; Flours</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
       </c>
       <c r="E20" t="n">
-        <v>25</v>
+        <v>387</v>
       </c>
       <c r="F20" t="n">
-        <v>55</v>
+        <v>180</v>
       </c>
       <c r="G20" t="n">
+        <v>350</v>
+      </c>
+      <c r="H20" t="n">
         <v>5</v>
       </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>LOW STOCK</t>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>IN STOCK</t>
         </is>
       </c>
     </row>
@@ -1112,29 +1212,34 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Active Dry Yeast</t>
+          <t>Hard Wheat Bread Flour</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="D21" t="n">
-        <v>42</v>
+          <t>Grains &amp; Flours</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
       </c>
       <c r="E21" t="n">
-        <v>18</v>
+        <v>341</v>
       </c>
       <c r="F21" t="n">
-        <v>35</v>
+        <v>450</v>
       </c>
       <c r="G21" t="n">
-        <v>5</v>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>IN STOCK</t>
+        <v>900</v>
+      </c>
+      <c r="H21" t="n">
+        <v>3</v>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>LOW STOCK</t>
         </is>
       </c>
     </row>
@@ -1146,27 +1251,32 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Baking Powder (Double Acting)</t>
+          <t>Purified Water</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="D22" t="n">
-        <v>58</v>
+          <t>Liquids</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
       </c>
       <c r="E22" t="n">
-        <v>25</v>
+        <v>2152</v>
       </c>
       <c r="F22" t="n">
-        <v>60</v>
+        <v>1000</v>
       </c>
       <c r="G22" t="n">
-        <v>4</v>
-      </c>
-      <c r="H22" t="inlineStr">
+        <v>2000</v>
+      </c>
+      <c r="H22" t="n">
+        <v>1</v>
+      </c>
+      <c r="I22" t="inlineStr">
         <is>
           <t>IN STOCK</t>
         </is>
@@ -1180,27 +1290,32 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Baking Soda</t>
+          <t>Cleaned Chicken Crop (Butse)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="D23" t="n">
-        <v>15</v>
+          <t>Meat &amp; Poultry</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
       </c>
       <c r="E23" t="n">
-        <v>20</v>
+        <v>39</v>
       </c>
       <c r="F23" t="n">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="G23" t="n">
-        <v>4</v>
-      </c>
-      <c r="H23" t="inlineStr">
+        <v>100</v>
+      </c>
+      <c r="H23" t="n">
+        <v>2</v>
+      </c>
+      <c r="I23" t="inlineStr">
         <is>
           <t>LOW STOCK</t>
         </is>
@@ -1214,29 +1329,34 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Iodized Fine Salt</t>
+          <t>Pork Skin with Back Fat</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="D24" t="n">
-        <v>71</v>
+          <t>Meat &amp; Poultry</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
       </c>
       <c r="E24" t="n">
-        <v>30</v>
+        <v>152</v>
       </c>
       <c r="F24" t="n">
-        <v>70</v>
+        <v>200</v>
       </c>
       <c r="G24" t="n">
-        <v>3</v>
-      </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>IN STOCK</t>
+        <v>400</v>
+      </c>
+      <c r="H24" t="n">
+        <v>2</v>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>LOW STOCK</t>
         </is>
       </c>
     </row>
@@ -1248,27 +1368,32 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Dark Chocolate Couverture (65%)</t>
+          <t>Raw Shelled Peanuts</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="D25" t="n">
-        <v>68</v>
+          <t>Nuts &amp; Seeds</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
       </c>
       <c r="E25" t="n">
-        <v>90</v>
+        <v>116</v>
       </c>
       <c r="F25" t="n">
-        <v>210</v>
+        <v>150</v>
       </c>
       <c r="G25" t="n">
+        <v>300</v>
+      </c>
+      <c r="H25" t="n">
         <v>5</v>
       </c>
-      <c r="H25" t="inlineStr">
+      <c r="I25" t="inlineStr">
         <is>
           <t>LOW STOCK</t>
         </is>
@@ -1282,27 +1407,32 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Milk Chocolate Chips</t>
+          <t>Toasted Sesame Seeds</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="D26" t="n">
-        <v>151</v>
+          <t>Nuts &amp; Seeds</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
       </c>
       <c r="E26" t="n">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="F26" t="n">
-        <v>160</v>
+        <v>30</v>
       </c>
       <c r="G26" t="n">
-        <v>4</v>
-      </c>
-      <c r="H26" t="inlineStr">
+        <v>60</v>
+      </c>
+      <c r="H26" t="n">
+        <v>5</v>
+      </c>
+      <c r="I26" t="inlineStr">
         <is>
           <t>IN STOCK</t>
         </is>
@@ -1316,27 +1446,32 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>White Chocolate Compound</t>
+          <t>Palm Cooking Oil</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="D27" t="n">
-        <v>40</v>
+          <t>Oils &amp; Fats</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
       </c>
       <c r="E27" t="n">
-        <v>55</v>
+        <v>526</v>
       </c>
       <c r="F27" t="n">
-        <v>130</v>
+        <v>700</v>
       </c>
       <c r="G27" t="n">
-        <v>4</v>
-      </c>
-      <c r="H27" t="inlineStr">
+        <v>1400</v>
+      </c>
+      <c r="H27" t="n">
+        <v>3</v>
+      </c>
+      <c r="I27" t="inlineStr">
         <is>
           <t>LOW STOCK</t>
         </is>
@@ -1350,29 +1485,34 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Alkalized Cocoa Powder</t>
+          <t>Pure Pork Lard</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="D28" t="n">
-        <v>41</v>
+          <t>Oils &amp; Fats</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
       </c>
       <c r="E28" t="n">
-        <v>55</v>
+        <v>217</v>
       </c>
       <c r="F28" t="n">
-        <v>135</v>
+        <v>100</v>
       </c>
       <c r="G28" t="n">
-        <v>5</v>
-      </c>
-      <c r="H28" t="inlineStr">
-        <is>
-          <t>LOW STOCK</t>
+        <v>200</v>
+      </c>
+      <c r="H28" t="n">
+        <v>4</v>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>IN STOCK</t>
         </is>
       </c>
     </row>
@@ -1384,27 +1524,32 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Pure Vanilla Extract</t>
+          <t>Refined Peanut Oil</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
+          <t>Oils &amp; Fats</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
           <t>L</t>
         </is>
       </c>
-      <c r="D29" t="n">
-        <v>29</v>
-      </c>
       <c r="E29" t="n">
-        <v>12</v>
+        <v>175</v>
       </c>
       <c r="F29" t="n">
-        <v>30</v>
+        <v>80</v>
       </c>
       <c r="G29" t="n">
-        <v>6</v>
-      </c>
-      <c r="H29" t="inlineStr">
+        <v>150</v>
+      </c>
+      <c r="H29" t="n">
+        <v>5</v>
+      </c>
+      <c r="I29" t="inlineStr">
         <is>
           <t>IN STOCK</t>
         </is>
@@ -1418,27 +1563,32 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Artificial Vanilla Flavoring</t>
+          <t>Fresh Carrots</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="D30" t="n">
-        <v>43</v>
+          <t>Produce / Agricultural</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
       </c>
       <c r="E30" t="n">
-        <v>18</v>
+        <v>133</v>
       </c>
       <c r="F30" t="n">
-        <v>42</v>
+        <v>60</v>
       </c>
       <c r="G30" t="n">
-        <v>3</v>
-      </c>
-      <c r="H30" t="inlineStr">
+        <v>120</v>
+      </c>
+      <c r="H30" t="n">
+        <v>2</v>
+      </c>
+      <c r="I30" t="inlineStr">
         <is>
           <t>IN STOCK</t>
         </is>
@@ -1452,27 +1602,32 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Ube Flavor Paste</t>
+          <t>Fresh Cassava Tubers</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="D31" t="n">
-        <v>33</v>
+          <t>Produce / Agricultural</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
       </c>
       <c r="E31" t="n">
-        <v>40</v>
+        <v>151</v>
       </c>
       <c r="F31" t="n">
-        <v>95</v>
+        <v>200</v>
       </c>
       <c r="G31" t="n">
-        <v>4</v>
-      </c>
-      <c r="H31" t="inlineStr">
+        <v>400</v>
+      </c>
+      <c r="H31" t="n">
+        <v>2</v>
+      </c>
+      <c r="I31" t="inlineStr">
         <is>
           <t>LOW STOCK</t>
         </is>
@@ -1486,27 +1641,32 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Pandan Extract Essence</t>
+          <t>Fresh Garlic</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="D32" t="n">
-        <v>9</v>
+          <t>Produce / Agricultural</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
       </c>
       <c r="E32" t="n">
-        <v>12</v>
+        <v>92</v>
       </c>
       <c r="F32" t="n">
-        <v>26</v>
+        <v>120</v>
       </c>
       <c r="G32" t="n">
-        <v>4</v>
-      </c>
-      <c r="H32" t="inlineStr">
+        <v>240</v>
+      </c>
+      <c r="H32" t="n">
+        <v>3</v>
+      </c>
+      <c r="I32" t="inlineStr">
         <is>
           <t>LOW STOCK</t>
         </is>
@@ -1520,27 +1680,32 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Ground Cinnamon Powder</t>
+          <t>Fresh Ginger</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="D33" t="n">
-        <v>39</v>
+          <t>Produce / Agricultural</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
       </c>
       <c r="E33" t="n">
-        <v>15</v>
+        <v>109</v>
       </c>
       <c r="F33" t="n">
-        <v>35</v>
+        <v>50</v>
       </c>
       <c r="G33" t="n">
-        <v>5</v>
-      </c>
-      <c r="H33" t="inlineStr">
+        <v>100</v>
+      </c>
+      <c r="H33" t="n">
+        <v>3</v>
+      </c>
+      <c r="I33" t="inlineStr">
         <is>
           <t>IN STOCK</t>
         </is>
@@ -1554,27 +1719,32 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Nutmeg Powder</t>
+          <t>Fresh Grated Coconut Meat</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="D34" t="n">
-        <v>13</v>
+          <t>Produce / Agricultural</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
       </c>
       <c r="E34" t="n">
-        <v>6</v>
+        <v>303</v>
       </c>
       <c r="F34" t="n">
-        <v>15</v>
+        <v>140</v>
       </c>
       <c r="G34" t="n">
-        <v>6</v>
-      </c>
-      <c r="H34" t="inlineStr">
+        <v>280</v>
+      </c>
+      <c r="H34" t="n">
+        <v>2</v>
+      </c>
+      <c r="I34" t="inlineStr">
         <is>
           <t>IN STOCK</t>
         </is>
@@ -1588,29 +1758,34 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Cheddar Cheese Block</t>
+          <t>Fresh Mature Coconut Meat</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="D35" t="n">
-        <v>50</v>
+          <t>Produce / Agricultural</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
       </c>
       <c r="E35" t="n">
-        <v>65</v>
+        <v>326</v>
       </c>
       <c r="F35" t="n">
-        <v>155</v>
+        <v>150</v>
       </c>
       <c r="G35" t="n">
-        <v>3</v>
-      </c>
-      <c r="H35" t="inlineStr">
-        <is>
-          <t>LOW STOCK</t>
+        <v>300</v>
+      </c>
+      <c r="H35" t="n">
+        <v>2</v>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>IN STOCK</t>
         </is>
       </c>
     </row>
@@ -1622,27 +1797,32 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Cream Cheese</t>
+          <t>Fresh Purple Yam Tubers</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="D36" t="n">
-        <v>58</v>
+          <t>Produce / Agricultural</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
       </c>
       <c r="E36" t="n">
-        <v>75</v>
+        <v>152</v>
       </c>
       <c r="F36" t="n">
-        <v>175</v>
+        <v>200</v>
       </c>
       <c r="G36" t="n">
+        <v>400</v>
+      </c>
+      <c r="H36" t="n">
         <v>3</v>
       </c>
-      <c r="H36" t="inlineStr">
+      <c r="I36" t="inlineStr">
         <is>
           <t>LOW STOCK</t>
         </is>
@@ -1656,27 +1836,32 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Grated Parmesan Cheese</t>
+          <t>Fresh Sweet Potato</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="D37" t="n">
-        <v>68</v>
+          <t>Produce / Agricultural</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
       </c>
       <c r="E37" t="n">
-        <v>30</v>
+        <v>220</v>
       </c>
       <c r="F37" t="n">
-        <v>70</v>
+        <v>100</v>
       </c>
       <c r="G37" t="n">
-        <v>4</v>
-      </c>
-      <c r="H37" t="inlineStr">
+        <v>200</v>
+      </c>
+      <c r="H37" t="n">
+        <v>3</v>
+      </c>
+      <c r="I37" t="inlineStr">
         <is>
           <t>IN STOCK</t>
         </is>
@@ -1690,27 +1875,32 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Quick-Melt Cheese</t>
+          <t>Green Raw Papaya</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="D38" t="n">
-        <v>122</v>
+          <t>Produce / Agricultural</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
       </c>
       <c r="E38" t="n">
-        <v>55</v>
+        <v>194</v>
       </c>
       <c r="F38" t="n">
-        <v>130</v>
+        <v>90</v>
       </c>
       <c r="G38" t="n">
-        <v>3</v>
-      </c>
-      <c r="H38" t="inlineStr">
+        <v>180</v>
+      </c>
+      <c r="H38" t="n">
+        <v>2</v>
+      </c>
+      <c r="I38" t="inlineStr">
         <is>
           <t>IN STOCK</t>
         </is>
@@ -1724,29 +1914,34 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Roasted Almond Slices</t>
+          <t>Pandan Leaves</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="D39" t="n">
-        <v>24</v>
+          <t>Produce / Agricultural</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
       </c>
       <c r="E39" t="n">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="F39" t="n">
-        <v>80</v>
+        <v>10</v>
       </c>
       <c r="G39" t="n">
-        <v>6</v>
-      </c>
-      <c r="H39" t="inlineStr">
-        <is>
-          <t>LOW STOCK</t>
+        <v>20</v>
+      </c>
+      <c r="H39" t="n">
+        <v>2</v>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>IN STOCK</t>
         </is>
       </c>
     </row>
@@ -1758,29 +1953,34 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Walnut Halves</t>
+          <t>Red Bell Peppers</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="D40" t="n">
-        <v>21</v>
+          <t>Produce / Agricultural</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
       </c>
       <c r="E40" t="n">
-        <v>25</v>
+        <v>67</v>
       </c>
       <c r="F40" t="n">
-        <v>65</v>
+        <v>30</v>
       </c>
       <c r="G40" t="n">
-        <v>6</v>
-      </c>
-      <c r="H40" t="inlineStr">
-        <is>
-          <t>LOW STOCK</t>
+        <v>60</v>
+      </c>
+      <c r="H40" t="n">
+        <v>3</v>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>IN STOCK</t>
         </is>
       </c>
     </row>
@@ -1792,29 +1992,34 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Desiccated Coconut (Medium)</t>
+          <t>Red Chili Peppers (Siling Labuyo)</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="D41" t="n">
-        <v>104</v>
+          <t>Produce / Agricultural</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
       </c>
       <c r="E41" t="n">
-        <v>45</v>
+        <v>14</v>
       </c>
       <c r="F41" t="n">
-        <v>105</v>
+        <v>15</v>
       </c>
       <c r="G41" t="n">
-        <v>4</v>
-      </c>
-      <c r="H41" t="inlineStr">
-        <is>
-          <t>IN STOCK</t>
+        <v>30</v>
+      </c>
+      <c r="H41" t="n">
+        <v>2</v>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>LOW STOCK</t>
         </is>
       </c>
     </row>
@@ -1826,27 +2031,32 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Black Sesame Seeds</t>
+          <t>Red Onions</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="D42" t="n">
-        <v>39</v>
+          <t>Produce / Agricultural</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
       </c>
       <c r="E42" t="n">
-        <v>18</v>
+        <v>219</v>
       </c>
       <c r="F42" t="n">
-        <v>40</v>
+        <v>100</v>
       </c>
       <c r="G42" t="n">
-        <v>5</v>
-      </c>
-      <c r="H42" t="inlineStr">
+        <v>200</v>
+      </c>
+      <c r="H42" t="n">
+        <v>3</v>
+      </c>
+      <c r="I42" t="inlineStr">
         <is>
           <t>IN STOCK</t>
         </is>
@@ -1860,27 +2070,32 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>White Sesame Seeds</t>
+          <t>Unripe Green Saba Bananas</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="D43" t="n">
-        <v>17</v>
+          <t>Produce / Agricultural</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
       </c>
       <c r="E43" t="n">
-        <v>22</v>
+        <v>339</v>
       </c>
       <c r="F43" t="n">
-        <v>52</v>
+        <v>450</v>
       </c>
       <c r="G43" t="n">
-        <v>4</v>
-      </c>
-      <c r="H43" t="inlineStr">
+        <v>900</v>
+      </c>
+      <c r="H43" t="n">
+        <v>2</v>
+      </c>
+      <c r="I43" t="inlineStr">
         <is>
           <t>LOW STOCK</t>
         </is>
@@ -1894,29 +2109,34 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Strawberry Jam Filling</t>
+          <t>Fresh Acetes Shrimp (Alamang)</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="D44" t="n">
-        <v>38</v>
+          <t>Seafood</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
       </c>
       <c r="E44" t="n">
-        <v>50</v>
+        <v>151</v>
       </c>
       <c r="F44" t="n">
-        <v>115</v>
+        <v>70</v>
       </c>
       <c r="G44" t="n">
-        <v>3</v>
-      </c>
-      <c r="H44" t="inlineStr">
-        <is>
-          <t>LOW STOCK</t>
+        <v>140</v>
+      </c>
+      <c r="H44" t="n">
+        <v>2</v>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>IN STOCK</t>
         </is>
       </c>
     </row>
@@ -1928,29 +2148,34 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Blueberry Fruit Filling</t>
+          <t>Fresh Bangus (Milkfish) Skin</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="D45" t="n">
-        <v>89</v>
+          <t>Seafood</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
       </c>
       <c r="E45" t="n">
-        <v>40</v>
+        <v>63</v>
       </c>
       <c r="F45" t="n">
-        <v>95</v>
+        <v>80</v>
       </c>
       <c r="G45" t="n">
-        <v>4</v>
-      </c>
-      <c r="H45" t="inlineStr">
-        <is>
-          <t>IN STOCK</t>
+        <v>160</v>
+      </c>
+      <c r="H45" t="n">
+        <v>2</v>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>LOW STOCK</t>
         </is>
       </c>
     </row>
@@ -1962,27 +2187,32 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Bavarian Cream Filling</t>
+          <t>Fresh Chiton Mollusk (Kibit)</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="D46" t="n">
-        <v>47</v>
+          <t>Seafood</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
       </c>
       <c r="E46" t="n">
-        <v>60</v>
+        <v>38</v>
       </c>
       <c r="F46" t="n">
-        <v>140</v>
+        <v>50</v>
       </c>
       <c r="G46" t="n">
-        <v>3</v>
-      </c>
-      <c r="H46" t="inlineStr">
+        <v>100</v>
+      </c>
+      <c r="H46" t="n">
+        <v>2</v>
+      </c>
+      <c r="I46" t="inlineStr">
         <is>
           <t>LOW STOCK</t>
         </is>
@@ -1996,27 +2226,32 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Pineapple Crushed (Canned)</t>
+          <t>Fresh Kabasi Fish</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="D47" t="n">
+          <t>Seafood</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="E47" t="n">
+        <v>89</v>
+      </c>
+      <c r="F47" t="n">
+        <v>40</v>
+      </c>
+      <c r="G47" t="n">
         <v>80</v>
       </c>
-      <c r="E47" t="n">
-        <v>35</v>
-      </c>
-      <c r="F47" t="n">
-        <v>85</v>
-      </c>
-      <c r="G47" t="n">
-        <v>4</v>
-      </c>
-      <c r="H47" t="inlineStr">
+      <c r="H47" t="n">
+        <v>2</v>
+      </c>
+      <c r="I47" t="inlineStr">
         <is>
           <t>IN STOCK</t>
         </is>
@@ -2030,27 +2265,32 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Cornstarch (Maizena)</t>
+          <t>Fresh Sapsap Fish</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="D48" t="n">
-        <v>114</v>
+          <t>Seafood</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
       </c>
       <c r="E48" t="n">
+        <v>112</v>
+      </c>
+      <c r="F48" t="n">
         <v>50</v>
       </c>
-      <c r="F48" t="n">
-        <v>125</v>
-      </c>
       <c r="G48" t="n">
-        <v>3</v>
-      </c>
-      <c r="H48" t="inlineStr">
+        <v>100</v>
+      </c>
+      <c r="H48" t="n">
+        <v>2</v>
+      </c>
+      <c r="I48" t="inlineStr">
         <is>
           <t>IN STOCK</t>
         </is>
@@ -2064,27 +2304,32 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Bread Improver (Enzyme)</t>
+          <t>Cheese Seasoning Powder</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="D49" t="n">
-        <v>9</v>
+          <t>Seasonings &amp; Powders</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
       </c>
       <c r="E49" t="n">
-        <v>10</v>
+        <v>29</v>
       </c>
       <c r="F49" t="n">
-        <v>22</v>
+        <v>35</v>
       </c>
       <c r="G49" t="n">
+        <v>70</v>
+      </c>
+      <c r="H49" t="n">
         <v>5</v>
       </c>
-      <c r="H49" t="inlineStr">
+      <c r="I49" t="inlineStr">
         <is>
           <t>LOW STOCK</t>
         </is>
@@ -2098,29 +2343,34 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Emulsifier Paste (Ovalette)</t>
+          <t>Coarse Rock Salt</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="D50" t="n">
-        <v>14</v>
+          <t>Seasonings / Salts</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
       </c>
       <c r="E50" t="n">
-        <v>15</v>
+        <v>323</v>
       </c>
       <c r="F50" t="n">
-        <v>35</v>
+        <v>150</v>
       </c>
       <c r="G50" t="n">
-        <v>5</v>
-      </c>
-      <c r="H50" t="inlineStr">
-        <is>
-          <t>LOW STOCK</t>
+        <v>300</v>
+      </c>
+      <c r="H50" t="n">
+        <v>4</v>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>IN STOCK</t>
         </is>
       </c>
     </row>
@@ -2132,27 +2382,32 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Calcium Propionate (Preservative)</t>
+          <t>Iodized Salt</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="D51" t="n">
-        <v>18</v>
+          <t>Seasonings / Salts</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
       </c>
       <c r="E51" t="n">
-        <v>8</v>
+        <v>431</v>
       </c>
       <c r="F51" t="n">
-        <v>18</v>
+        <v>200</v>
       </c>
       <c r="G51" t="n">
-        <v>6</v>
-      </c>
-      <c r="H51" t="inlineStr">
+        <v>400</v>
+      </c>
+      <c r="H51" t="n">
+        <v>4</v>
+      </c>
+      <c r="I51" t="inlineStr">
         <is>
           <t>IN STOCK</t>
         </is>
@@ -2166,27 +2421,32 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Liquid Glucose Syrup</t>
+          <t>Dried Bay Leaves (Laurel)</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="D52" t="n">
-        <v>99</v>
+          <t>Spices &amp; Seasonings</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
       </c>
       <c r="E52" t="n">
-        <v>45</v>
+        <v>19</v>
       </c>
       <c r="F52" t="n">
-        <v>105</v>
+        <v>8</v>
       </c>
       <c r="G52" t="n">
-        <v>4</v>
-      </c>
-      <c r="H52" t="inlineStr">
+        <v>15</v>
+      </c>
+      <c r="H52" t="n">
+        <v>7</v>
+      </c>
+      <c r="I52" t="inlineStr">
         <is>
           <t>IN STOCK</t>
         </is>
@@ -2200,27 +2460,32 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Honey Pure Bee</t>
+          <t>Dried Red Chili Flakes</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="D53" t="n">
-        <v>19</v>
+          <t>Spices &amp; Seasonings</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
       </c>
       <c r="E53" t="n">
+        <v>12</v>
+      </c>
+      <c r="F53" t="n">
+        <v>12</v>
+      </c>
+      <c r="G53" t="n">
         <v>25</v>
       </c>
-      <c r="F53" t="n">
-        <v>58</v>
-      </c>
-      <c r="G53" t="n">
-        <v>5</v>
-      </c>
-      <c r="H53" t="inlineStr">
+      <c r="H53" t="n">
+        <v>6</v>
+      </c>
+      <c r="I53" t="inlineStr">
         <is>
           <t>LOW STOCK</t>
         </is>
@@ -2234,27 +2499,32 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Matcha Green Tea Powder</t>
+          <t>Garlic Powder</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="D54" t="n">
-        <v>13</v>
+          <t>Spices &amp; Seasonings</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
       </c>
       <c r="E54" t="n">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F54" t="n">
-        <v>38</v>
+        <v>25</v>
       </c>
       <c r="G54" t="n">
-        <v>7</v>
-      </c>
-      <c r="H54" t="inlineStr">
+        <v>50</v>
+      </c>
+      <c r="H54" t="n">
+        <v>5</v>
+      </c>
+      <c r="I54" t="inlineStr">
         <is>
           <t>LOW STOCK</t>
         </is>
@@ -2268,27 +2538,32 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Red Food Coloring (Gel)</t>
+          <t>Ground Black Pepper</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="D55" t="n">
-        <v>16</v>
+          <t>Spices &amp; Seasonings</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
       </c>
       <c r="E55" t="n">
+        <v>91</v>
+      </c>
+      <c r="F55" t="n">
+        <v>40</v>
+      </c>
+      <c r="G55" t="n">
+        <v>80</v>
+      </c>
+      <c r="H55" t="n">
         <v>5</v>
       </c>
-      <c r="F55" t="n">
-        <v>12</v>
-      </c>
-      <c r="G55" t="n">
-        <v>4</v>
-      </c>
-      <c r="H55" t="inlineStr">
+      <c r="I55" t="inlineStr">
         <is>
           <t>IN STOCK</t>
         </is>
@@ -2302,27 +2577,32 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Yellow Food Coloring (Gel)</t>
+          <t>White Pepper Powder</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="D56" t="n">
-        <v>17</v>
+          <t>Spices &amp; Seasonings</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
       </c>
       <c r="E56" t="n">
+        <v>43</v>
+      </c>
+      <c r="F56" t="n">
+        <v>20</v>
+      </c>
+      <c r="G56" t="n">
+        <v>40</v>
+      </c>
+      <c r="H56" t="n">
         <v>5</v>
       </c>
-      <c r="F56" t="n">
-        <v>12</v>
-      </c>
-      <c r="G56" t="n">
-        <v>4</v>
-      </c>
-      <c r="H56" t="inlineStr">
+      <c r="I56" t="inlineStr">
         <is>
           <t>IN STOCK</t>
         </is>
@@ -2336,27 +2616,32 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Green Food Coloring (Gel)</t>
+          <t>Whole Black Peppercorns</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="D57" t="n">
-        <v>3</v>
+          <t>Spices &amp; Seasonings</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
       </c>
       <c r="E57" t="n">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="F57" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="G57" t="n">
-        <v>4</v>
-      </c>
-      <c r="H57" t="inlineStr">
+        <v>40</v>
+      </c>
+      <c r="H57" t="n">
+        <v>6</v>
+      </c>
+      <c r="I57" t="inlineStr">
         <is>
           <t>LOW STOCK</t>
         </is>
@@ -2370,29 +2655,34 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Instant Coffee Powder</t>
+          <t>Muscovado Brown Sugar</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="D58" t="n">
-        <v>17</v>
+          <t>Sweeteners</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
       </c>
       <c r="E58" t="n">
-        <v>22</v>
+        <v>475</v>
       </c>
       <c r="F58" t="n">
-        <v>48</v>
+        <v>220</v>
       </c>
       <c r="G58" t="n">
+        <v>450</v>
+      </c>
+      <c r="H58" t="n">
         <v>4</v>
       </c>
-      <c r="H58" t="inlineStr">
-        <is>
-          <t>LOW STOCK</t>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>IN STOCK</t>
         </is>
       </c>
     </row>
@@ -2404,29 +2694,34 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Rolled Oats (Old Fashioned)</t>
+          <t>Panutsa Cane Sugar</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="D59" t="n">
-        <v>66</v>
+          <t>Sweeteners</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
       </c>
       <c r="E59" t="n">
-        <v>30</v>
+        <v>99</v>
       </c>
       <c r="F59" t="n">
-        <v>75</v>
+        <v>130</v>
       </c>
       <c r="G59" t="n">
+        <v>260</v>
+      </c>
+      <c r="H59" t="n">
         <v>4</v>
       </c>
-      <c r="H59" t="inlineStr">
-        <is>
-          <t>IN STOCK</t>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>LOW STOCK</t>
         </is>
       </c>
     </row>
@@ -2438,29 +2733,34 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Golden Raisins Seedless</t>
+          <t>Refined White Sugar</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="D60" t="n">
-        <v>62</v>
+          <t>Sweeteners</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
       </c>
       <c r="E60" t="n">
-        <v>28</v>
+        <v>565</v>
       </c>
       <c r="F60" t="n">
-        <v>65</v>
+        <v>750</v>
       </c>
       <c r="G60" t="n">
-        <v>5</v>
-      </c>
-      <c r="H60" t="inlineStr">
-        <is>
-          <t>IN STOCK</t>
+        <v>1500</v>
+      </c>
+      <c r="H60" t="n">
+        <v>3</v>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>LOW STOCK</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(dataset): configure realistic Out of Stock situation on 4 key raw materials
</commit_message>
<xml_diff>
--- a/DATASETS/ACTUAL_DATA_2026_YTD/RMIMS_59_RAW_MATERIALS_CATALOG.xlsx
+++ b/DATASETS/ACTUAL_DATA_2026_YTD/RMIMS_59_RAW_MATERIALS_CATALOG.xlsx
@@ -1343,7 +1343,7 @@
         </is>
       </c>
       <c r="E24" t="n">
-        <v>152</v>
+        <v>0</v>
       </c>
       <c r="F24" t="n">
         <v>200</v>
@@ -1356,7 +1356,7 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>LOW STOCK</t>
+          <t>OUT OF STOCK</t>
         </is>
       </c>
     </row>
@@ -1655,7 +1655,7 @@
         </is>
       </c>
       <c r="E32" t="n">
-        <v>92</v>
+        <v>0</v>
       </c>
       <c r="F32" t="n">
         <v>120</v>
@@ -1668,7 +1668,7 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>LOW STOCK</t>
+          <t>OUT OF STOCK</t>
         </is>
       </c>
     </row>
@@ -2084,7 +2084,7 @@
         </is>
       </c>
       <c r="E43" t="n">
-        <v>339</v>
+        <v>0</v>
       </c>
       <c r="F43" t="n">
         <v>450</v>
@@ -2097,7 +2097,7 @@
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>LOW STOCK</t>
+          <t>OUT OF STOCK</t>
         </is>
       </c>
     </row>
@@ -2201,7 +2201,7 @@
         </is>
       </c>
       <c r="E46" t="n">
-        <v>38</v>
+        <v>0</v>
       </c>
       <c r="F46" t="n">
         <v>50</v>
@@ -2214,7 +2214,7 @@
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>LOW STOCK</t>
+          <t>OUT OF STOCK</t>
         </is>
       </c>
     </row>

</xml_diff>